<commit_message>
paper run 2026-09-28 18:46
</commit_message>
<xml_diff>
--- a/reports/2026-09-28.xlsx
+++ b/reports/2026-09-28.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -606,7 +606,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-28T04:12:39.156369+00:00</t>
+          <t>2026-09-28T09:26:17.998714+00:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -616,26 +616,26 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="D5" t="n">
         <v>15</v>
       </c>
       <c r="E5" t="n">
-        <v>0.6</v>
+        <v>0.52</v>
       </c>
       <c r="F5" t="n">
-        <v>10.8</v>
+        <v>15.6</v>
       </c>
       <c r="G5" t="n">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="H5" t="n">
-        <v>0.796</v>
+        <v>0.765</v>
       </c>
       <c r="I5" t="n">
-        <v>0.00144</v>
+        <v>-0.00132</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -643,7 +643,179 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>7.2</v>
+        <v>14.4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-28T13:53:57.933748+00:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="F6" t="n">
+        <v>51.73</v>
+      </c>
+      <c r="G6" t="n">
+        <v>84.81</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.777</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.00131</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>33.08</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-28T14:26:38.456363+00:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>15</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="F7" t="n">
+        <v>6.71</v>
+      </c>
+      <c r="G7" t="n">
+        <v>11</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.831</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.00326</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>-6.71</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-28T14:42:14.475991+00:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="F8" t="n">
+        <v>12.77</v>
+      </c>
+      <c r="G8" t="n">
+        <v>20.93</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.8129999999999999</v>
+      </c>
+      <c r="I8" t="n">
+        <v>-0.00228</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>8.16</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-28T17:11:36.518039+00:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>15</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.5116000000000001</v>
+      </c>
+      <c r="F9" t="n">
+        <v>23.43</v>
+      </c>
+      <c r="G9" t="n">
+        <v>45.79</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.788</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.00187</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>22.36</v>
       </c>
     </row>
   </sheetData>
@@ -657,7 +829,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -679,7 +851,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
@@ -689,7 +861,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -699,7 +871,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -709,7 +881,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="6">
@@ -719,7 +891,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>117.66</v>
+        <v>181.75</v>
       </c>
     </row>
     <row r="7">
@@ -729,7 +901,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>117.66</v>
+        <v>188.46</v>
       </c>
     </row>
     <row r="8">
@@ -739,7 +911,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>-6.71</v>
       </c>
     </row>
     <row r="9">
@@ -749,7 +921,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>99</v>
+        <v>28.09</v>
       </c>
     </row>
     <row r="10">
@@ -759,7 +931,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2051.1</v>
+        <v>2115.19</v>
       </c>
     </row>
     <row r="12">
@@ -810,16 +982,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="C15" t="n">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="D15" t="n">
-        <v>221.48</v>
+        <v>1207.33</v>
       </c>
       <c r="E15" t="n">
-        <v>107.54</v>
+        <v>145.75</v>
       </c>
     </row>
     <row r="16">
@@ -829,16 +1001,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C16" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D16" t="n">
-        <v>269.21</v>
+        <v>494.86</v>
       </c>
       <c r="E16" t="n">
-        <v>10.12</v>
+        <v>43.2</v>
       </c>
     </row>
     <row r="17">
@@ -855,16 +1027,16 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D18" t="n">
-        <v>166.54</v>
+        <v>197.38</v>
       </c>
       <c r="E18" t="n">
-        <v>100.34</v>
+        <v>133.42</v>
       </c>
     </row>
     <row r="19">
@@ -874,13 +1046,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D19" t="n">
-        <v>149.04</v>
+        <v>381.74</v>
       </c>
       <c r="E19" t="n">
         <v>10.12</v>
@@ -893,16 +1065,16 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C20" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D20" t="n">
-        <v>118.51</v>
+        <v>343.04</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>8.16</v>
       </c>
     </row>
     <row r="21">
@@ -912,16 +1084,16 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="C21" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D21" t="n">
-        <v>56.6</v>
+        <v>780.03</v>
       </c>
       <c r="E21" t="n">
-        <v>7.2</v>
+        <v>37.25</v>
       </c>
     </row>
     <row r="22">
@@ -938,16 +1110,16 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="C23" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="D23" t="n">
-        <v>237.81</v>
+        <v>983.3200000000001</v>
       </c>
       <c r="E23" t="n">
-        <v>100.34</v>
+        <v>137.1</v>
       </c>
     </row>
     <row r="24">
@@ -957,13 +1129,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C24" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D24" t="n">
-        <v>337.34</v>
+        <v>381.92</v>
       </c>
       <c r="E24" t="n">
         <v>17.32</v>
@@ -976,16 +1148,16 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D25" t="n">
-        <v>-84.45999999999999</v>
+        <v>336.95</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>34.53</v>
       </c>
     </row>
     <row r="26">
@@ -1002,13 +1174,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D27" t="n">
-        <v>94.33</v>
+        <v>300.84</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
@@ -1021,13 +1193,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="C28" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="D28" t="n">
-        <v>85.73</v>
+        <v>876.3200000000001</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
@@ -1040,16 +1212,16 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C29" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D29" t="n">
-        <v>310.63</v>
+        <v>525.03</v>
       </c>
       <c r="E29" t="n">
-        <v>117.66</v>
+        <v>188.95</v>
       </c>
     </row>
     <row r="31">
@@ -1088,13 +1260,13 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D34" t="n">
-        <v>100.34</v>
+        <v>133.42</v>
       </c>
     </row>
     <row r="35">
@@ -1116,115 +1288,115 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" t="n">
+        <v>8.16</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>XRP</t>
         </is>
       </c>
-      <c r="B36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C36" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" t="n">
-        <v>7.2</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+      <c r="B37" t="n">
+        <v>3</v>
+      </c>
+      <c r="C37" t="n">
+        <v>2</v>
+      </c>
+      <c r="D37" t="n">
+        <v>30.05</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>15m</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>3</v>
-      </c>
-      <c r="C39" t="n">
-        <v>3</v>
-      </c>
-      <c r="D39" t="n">
-        <v>107.54</v>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>6</v>
+      </c>
+      <c r="C40" t="n">
+        <v>5</v>
+      </c>
+      <c r="D40" t="n">
+        <v>138.55</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>5m</t>
         </is>
       </c>
-      <c r="B40" t="n">
-        <v>1</v>
-      </c>
-      <c r="C40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D40" t="n">
-        <v>10.12</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+      <c r="B41" t="n">
+        <v>2</v>
+      </c>
+      <c r="C41" t="n">
+        <v>2</v>
+      </c>
+      <c r="D41" t="n">
+        <v>43.2</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>00</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>1</v>
-      </c>
-      <c r="C43" t="n">
-        <v>1</v>
-      </c>
-      <c r="D43" t="n">
-        <v>10.12</v>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>00</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1234,13 +1406,13 @@
         <v>1</v>
       </c>
       <c r="D44" t="n">
-        <v>67.04000000000001</v>
+        <v>10.12</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1250,13 +1422,13 @@
         <v>1</v>
       </c>
       <c r="D45" t="n">
-        <v>33.3</v>
+        <v>67.04000000000001</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1266,67 +1438,77 @@
         <v>1</v>
       </c>
       <c r="D46" t="n">
-        <v>7.2</v>
+        <v>33.3</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
+        <v>14.4</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="n">
+        <v>33.08</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B49" t="n">
         <v>2</v>
       </c>
       <c r="C49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D49" t="n">
-        <v>100.34</v>
+        <v>1.45</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D50" t="n">
-        <v>17.32</v>
+        <v>22.36</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>По силе движения</t>
+          <t>По цене входа</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1348,87 +1530,189 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C53" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D53" t="n">
-        <v>100.34</v>
+        <v>137.1</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B54" t="n">
+        <v>1</v>
+      </c>
+      <c r="C54" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" t="n">
+        <v>10.12</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>3</v>
+      </c>
+      <c r="C55" t="n">
         <v>2</v>
       </c>
-      <c r="C54" t="n">
-        <v>2</v>
-      </c>
-      <c r="D54" t="n">
-        <v>17.32</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+      <c r="D55" t="n">
+        <v>34.53</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="B57" t="n">
-        <v>1</v>
-      </c>
-      <c r="C57" t="n">
-        <v>1</v>
-      </c>
-      <c r="D57" t="n">
-        <v>33.3</v>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>2</v>
+      </c>
+      <c r="C58" t="n">
+        <v>2</v>
+      </c>
+      <c r="D58" t="n">
+        <v>100.34</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>3</v>
+      </c>
+      <c r="C59" t="n">
+        <v>3</v>
+      </c>
+      <c r="D59" t="n">
+        <v>57.6</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>1</v>
+      </c>
+      <c r="C60" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" t="n">
+        <v>22.36</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>0.20%+</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>2</v>
+      </c>
+      <c r="C61" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" t="n">
+        <v>1.45</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>3</v>
+      </c>
+      <c r="C64" t="n">
+        <v>3</v>
+      </c>
+      <c r="D64" t="n">
+        <v>55.86</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B58" t="n">
-        <v>3</v>
-      </c>
-      <c r="C58" t="n">
-        <v>3</v>
-      </c>
-      <c r="D58" t="n">
-        <v>84.36</v>
+      <c r="B65" t="n">
+        <v>5</v>
+      </c>
+      <c r="C65" t="n">
+        <v>4</v>
+      </c>
+      <c r="D65" t="n">
+        <v>125.89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>